<commit_message>
PHEVs qualify for ACC II
</commit_message>
<xml_diff>
--- a/InputData/trans/VTQaZ/Veh Techs Qualifying as ZEVs.xlsx
+++ b/InputData/trans/VTQaZ/Veh Techs Qualifying as ZEVs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\trans\VTQaZ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-maryland\InputData\trans\VTQaZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2410B116-F72B-481A-8955-3426D2F171F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC94D9DB-C3E7-45C9-B7E6-287A02DA6B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23640" xr2:uid="{7166B4F5-29DF-47A7-8501-7E54D22AC689}"/>
+    <workbookView xWindow="59325" yWindow="1665" windowWidth="24480" windowHeight="13800" activeTab="1" xr2:uid="{7166B4F5-29DF-47A7-8501-7E54D22AC689}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -440,14 +440,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C5140B-A3FA-4DAF-B6D3-27BA9BD40705}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -467,12 +467,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AF8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -570,7 +570,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -766,7 +766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1012,55 +1012,55 @@
         <v>1</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>

</xml_diff>